<commit_message>
Note Fieldglass dates used and evidence limitations in final conclusions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuGGWCwfLoBwzBBn34Y
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,6 +117,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -820,7 +823,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016501 OPEN 2024-01-01 to 2027-02-28 - active contractor; clears E2.</t>
+          <t>Worker SANWK00016501 OPEN 2024-01-01 to 2027-02-28 - active contractor; clears E2. Current work order SANWO00017798 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -875,7 +878,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016508 OPEN 2024-01-01 to 2027-02-28 - covers both decision dates.</t>
+          <t>Worker SANWK00016508 OPEN 2024-01-01 to 2027-02-28 - covers both decision dates. Current work order SANWO00017799 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -930,7 +933,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016502 OPEN 2024-01-01 to 2027-02-28.</t>
+          <t>Worker SANWK00016502 OPEN 2024-01-01 to 2027-02-28. Current work order SANWO00017797 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -985,7 +988,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016503 OPEN 2024-01-01 to 2027-02-28.</t>
+          <t>Worker SANWK00016503 OPEN 2024-01-01 to 2027-02-28. Current work order SANWO00017800 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1040,7 +1043,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016311 OPEN 2023-12-28 to 2027-02-28 - not terminated; does not explain the disablement.</t>
+          <t>Worker SANWK00016311 OPEN 2023-12-28 to 2027-02-28 - not terminated; does not explain the disablement. Current work order SANWO00017821 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1095,7 +1098,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Worker SANWK00016313 OPEN 2023-12-28 to 2027-02-28 - not terminated; does not explain the disablement.</t>
+          <t>Worker SANWK00016313 OPEN 2023-12-28 to 2027-02-28 - not terminated; does not explain the disablement. Current work order SANWO00017820 (Rev.18) Confirmed 2026-09-29 to 2027-02-28 - starts after the decision dates; continuity relies on the Open worker record period.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1137,6 +1140,20 @@
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Codes: A5 = appropriateness of approved access; A6 = revocation within SLA and sustained; E1 = AD disabled account approved; E2 = IAMS termination date; E3 = revoked access re-granted without approved request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Fieldglass evidence used: BSI Procurement email (Ana Belloso, 10/29/2026 13:52 UTC), screenshots image001-006. Dates used: Worker record status Open and period (2024-01-01 / 2023-12-28 to 2027-02-28) tested against decision dates 8/28/2025 and 4/30/2026; prior closed records 2023-10-08 to 2023-12-31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Fieldglass limitation: screenshots are search-result views with no report date/parameters, no extension history or approvers, and no status-as-of 8/28/2025, 4/30/2026 or April 2026 gap confirmation as requested on 10/14/2026; current work orders start 2026-09-29. Follow-up: request the worker 'Go to Details' view with work order revision history (Rev.0-Rev.18).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add process owner explanation and assessment columns to final conclusions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuGGWCwfLoBwzBBn34Y
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conclusions'!$A$4:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conclusions'!$A$4:$M$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,9 +117,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -496,9 +493,11 @@
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,15 +557,25 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>Process owner explanation</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Assessment of process owner explanation</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
           <t>Conclusion</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>What would change it</t>
         </is>
@@ -611,17 +620,27 @@
           <t>A6 (removal not sustained); A5-E3 (re-grant without request)</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Response (C7.Sample.xlsx) showed the account in the 2026 Q2 SOX Manager (rows 98-100) and CyberArk Manager (431-433) certifications, all Approved by Borges, Dayam, and AD enabled on 10/10/2026. No removal date, Netwrix log, ServiceNow ticket or explanation for the re-grant was provided. Process owner position: SanIAM shows no change / mover / leaver events.</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Not accepted. The response confirms the access is still held and was re-approved; it does not evidence an approved request for the re-grant after the 9/2/2025 removal. Exception stands.</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Revocation was timely but did not stay in place, and the re-granted access was approved without a request. E2 (IAMS term 12/31/2024) also unresolved - no Fieldglass evidence for this account.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Approved ServiceNow request + Netwrix 'member added' event for the re-grant; Fieldglass record.</t>
         </is>
@@ -666,17 +685,27 @@
           <t>A6; A5-E3; identity not correlated to HR (SUS.IAMS.4.2.1.1, 4.2.5.6)</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Response showed 2026 Q2 SOX Manager (140-142) and CyberArk Manager (467-468) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Not accepted. Re-approval in 2026 Q2 confirms the removal was not sustained. Exception stands.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Removal not sustained; re-grant and new ISEAdmin membership approved without requests; account not linked to an HR identity in SanIAM.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Requests + approvals for the re-grant and ISEAdmin add; correlate to SanIAM identity.</t>
         </is>
@@ -721,17 +750,27 @@
           <t>A6; A5-E3; identity not correlated to HR</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Response showed 2026 Q2 SOX Manager (143-145) and CyberArk Manager (469-471) rows Approved and AD enabled 10/10/2026. No re-grant request, Netwrix event or explanation provided; no explanation for the uncorrelated identity or the ISEAdmin add.</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Not accepted. Exception stands.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Removal not sustained; re-grant and new ISEAdmin membership approved without requests; account not linked to an HR identity.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Requests + approvals for the re-grant and ISEAdmin add; correlate to SanIAM identity.</t>
         </is>
@@ -776,17 +815,27 @@
           <t>A6; A5-E3</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Response showed 2026 Q2 SOX Manager (110-112) and CyberArk Manager (443-445) rows Approved and AD enabled 10/10/2026. No re-grant request or Netwrix event provided.</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Not accepted. Exception stands.</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Revocation timely but not sustained; re-grant approved without a request.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Approved ServiceNow request + Netwrix 'member added' event for the re-grant.</t>
         </is>
@@ -831,17 +880,27 @@
           <t>A5-E1 (disabled account approved) - SUS.IAMS.4.2.5.1, 4.2.5.7, 4.2.3.1</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>(1) 'If the access is approved, what SLA is being measured? The SLA only starts if the access is revoked.' (2) The consultants were extended - that is why they were certified in 2025 and 2026. (3) SanIAM shows no change, mover or leaver events. Fieldglass provided 10/29/2026 (worker SANWK00016501 Open 2024-01-01 to 2027-02-28). No explanation for why the disabled account keeps admin access.</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED - A6 N/A, no SLA exception. (2) SUPPORTED by Fieldglass - E2 cleared. (3) Does not explain approving an account disabled in AD and unused since 10/15/2023. A5-E1 exception stands.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Fieldglass shows he is an active contractor, but privileged admin access unused for ~2 years on a disabled account is not valid or needed (4.2.5.1); inactive accounts must be disabled or removed (4.2.3.1). The reviewer should have revoked it - exception in both samples.</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Recommend revocation; unlikely to clear.</t>
         </is>
@@ -886,17 +945,27 @@
           <t>E2 cleared - SUS.IAMS.4.2.1.1 (HR/Fieldglass authoritative), 4.2.5.6</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>(1) SLA only applies to revoked access. (2) Consultant contract was extended - that is why the account was certified. (3) No change / mover / leaver events in SanIAM. Fieldglass provided 10/29/2026 (worker SANWK00016508 Open 2024-01-01 to 2027-02-28; buyer ref 100531049 = SanIAM identity).</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED - A6 N/A. (2) SUPPORTED by Fieldglass - active on 8/28/2025 and 4/30/2026; IAMS 12/31/2024 is stale. Explanation accepted - no exception.</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Fieldglass shows an open engagement on both decision dates, so 12/31/2024 is stale SanIAM data, not a termination. Active, enabled account approved by the line manager (4.2.5.6). No exception.</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -941,17 +1010,27 @@
           <t>E2 cleared - SUS.IAMS.4.2.1.1, 4.2.5.6</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016502 Open 2024-01-01 to 2027-02-28; buyer ref 100531050 = SanIAM identity).</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED. (2) SUPPORTED by Fieldglass. Explanation accepted - no exception.</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Fieldglass clears the termination-date issue; approved access of an active, enabled contractor in both samples. No exception.</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -996,17 +1075,27 @@
           <t>E2 cleared - SUS.IAMS.4.2.1.1, 4.2.5.6</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016503 Open 2024-01-01 to 2027-02-28; buyer ref 100531051 = SanIAM identity).</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED. (2) SUPPORTED by Fieldglass. Explanation accepted - no exception.</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Fieldglass clears the termination-date issue; approved access of an active, enabled contractor in both samples. No exception.</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -1051,17 +1140,27 @@
           <t>A5-E1 (2026 Q1) - SUS.IAMS.4.2.5.1, 4.2.5.7; re-enable 4.2.3.4</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016311 Open 2023-12-28 to 2027-02-28; buyer ref 100592069 = SanIAM identity). No explanation for the 4/2/2026 AD disablement or the re-enable by 10/10/2026.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain approval on 4/30/2026 of an account disabled since 4/2/2026, or the unevidenced re-enable. A5-E1 exception stands for 2026 Q1.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>2025 Q3 passes. 2026 Q1 fails: privileged access approved on an account disabled since 4/2/2026; the later re-enable is unevidenced.</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Reason for the 4/2-4/3/2026 disablement of 9 contractor accounts + approved re-enable request could reduce to an observation.</t>
         </is>
@@ -1106,17 +1205,27 @@
           <t>A5-E1 (2026 Q1) - SUS.IAMS.4.2.5.1, 4.2.5.7, 4.2.3.4; 4.2.1.1 (AD not synced with HR)</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>(1) SLA only applies to revoked access. (2) Contract extended. (3) No change / mover / leaver events. Fieldglass provided (worker SANWK00016313 Open 2023-12-28 to 2027-02-28; buyer ref 100592068 = SanIAM identity). No explanation for the 4/3/2026 disablement, the re-enable, or the blank AD employeeNumber.</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>(1) AGREED - A6 N/A. (2) SUPPORTED - E2 cleared; 2025 Q3 passes. (3) Does not explain the 2026 Q1 approval of a disabled account or the re-enable. A5-E1 exception stands for 2026 Q1.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>2025 Q3 passes. 2026 Q1 fails: access approved on an account disabled since 4/3/2026; re-enable unevidenced; blank employeeNumber.</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Same as MIA25249; also populate employeeNumber.</t>
         </is>
@@ -1139,28 +1248,35 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>Process owner positions (walkthrough 3_Attribute Matrix table C and R7): (1) SLA applies only to revoked access - AGREED; (2) consultants were extended - SUPPORTED by Fieldglass 10/29/2026; (3) SanIAM shows no change / mover / leaver events - supports (2) but does not explain AD-disabled approvals or re-grants. Response file: BSI.IT.27.C7_E07_C7.Sample.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
           <t>Codes: A5 = appropriateness of approved access; A6 = revocation within SLA and sustained; E1 = AD disabled account approved; E2 = IAMS termination date; E3 = revoked access re-granted without approved request.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Fieldglass evidence used: BSI Procurement email (Ana Belloso, 10/29/2026 13:52 UTC), screenshots image001-006. Dates used: Worker record status Open and period (2024-01-01 / 2023-12-28 to 2027-02-28) tested against decision dates 8/28/2025 and 4/30/2026; prior closed records 2023-10-08 to 2023-12-31.</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Fieldglass limitation: screenshots are search-result views with no report date/parameters, no extension history or approvers, and no status-as-of 8/28/2025, 4/30/2026 or April 2026 gap confirmation as requested on 10/14/2026; current work orders start 2026-09-29. Follow-up: request the worker 'Go to Details' view with work order revision history (Rev.0-Rev.18).</t>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fieldglass evidence used: BSI Procurement email (Ana Belloso, 10/29/2026 13:52 UTC), screenshots image001-006. Worker record Open periods tested against decision dates 8/28/2025 and 4/30/2026. Fieldglass buyer references (100531048-51, 100592068-69) match the SanIAM identities in the management SAMPLE tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fieldglass limitation: search-result screenshots with no report date/parameters, extension history/approvers, or status-as-of-date / April 2026 gap confirmation; current work orders start 2026-09-29. Follow-up: request the worker 'Go to Details' view with work order revision history (Rev.0-Rev.18).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K14"/>
+  <autoFilter ref="A4:M14"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add policy basis column with quoted IAM Standard and PAM Procedure text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuGGWCwfLoBwzBBn34Y
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
+++ b/BSI.IT.27.C7_Final_Conclusions_10_Accounts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conclusions'!$A$4:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conclusions'!$A$4:$N$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +48,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F6000"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,6 +127,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -496,8 +512,9 @@
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="95" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -570,12 +587,17 @@
           <t>Conclusion</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Policy basis - why it passes / fails (with policy text)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>What would change it</t>
         </is>
@@ -635,12 +657,24 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: The 2025 Q3 removal met the 30-business-day SLA (4.2.5.21), but PAM Proc. 4.1.1 C4 and 4.2 require that revoked access stays removed and that retained access is escalated - it was back in AD by 11/25/2025 with no escalation. Under 4.2.5.7 the manager's denial means access is denied; giving it back required a new documented request, manager validation and second-level approval (4.2.3.4). None exists, yet the access was approved again on 4/30/2026.
+Also: IAMS termination date 12/31/2024 not supported by HR/Fieldglass evidence (4.2.1.1).
+IAM Std v10.0 SUS.IAMS.4.2.5.21 (p.22): "Any revocation of privileged access rights resulting from the privileged access review outcomes shall be completed within 30 business days of the close of the review."
+PAM Procedure v2.0 sec. 4.1.1 C4 (p.6): "When the ServiceNow ticket is closed, the PAM Team confirms that access is de-provisioned correctly."
+PAM Procedure v2.0 sec. 4.2 (p.7): "If PAM US Team identifies that a user whose access was rejected during a quarterly certification but maintained their privileges this finding will be escalated to senior management if the issue is not remediated."
+SUS.IAMS.4.2.5.7 (p.18): "Access is denied if any of the minimum required reviewers (workforce member's management ...) deny access to a workforce member."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Revocation was timely but did not stay in place, and the re-granted access was approved without a request. E2 (IAMS term 12/31/2024) also unresolved - no Fieldglass evidence for this account.</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Approved ServiceNow request + Netwrix 'member added' event for the re-grant; Fieldglass record.</t>
         </is>
@@ -700,12 +734,25 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: The 2025 Q3 removal met the 30-business-day SLA (4.2.5.21), but PAM Proc. 4.1.1 C4 and 4.2 require that revoked access stays removed and that retained access is escalated - it was back in AD by 11/25/2025 with no escalation. Under 4.2.5.7 the manager's denial means access is denied; giving it back required a new documented request, manager validation and second-level approval (4.2.3.4). None exists, yet the access was approved again on 4/30/2026.
+Also: the account is not correlated to an HR identity - 4.2.1.1 requires accounts synchronized with HR and 4.2.5.6 requires Application Owner attestation of uncorrelated accounts; the new ISEAdmin membership has no request (4.2.3.4).
+IAM Std v10.0 SUS.IAMS.4.2.5.21 (p.22): "Any revocation of privileged access rights resulting from the privileged access review outcomes shall be completed within 30 business days of the close of the review."
+PAM Procedure v2.0 sec. 4.1.1 C4 (p.6): "When the ServiceNow ticket is closed, the PAM Team confirms that access is de-provisioned correctly."
+PAM Procedure v2.0 sec. 4.2 (p.7): "If PAM US Team identifies that a user whose access was rejected during a quarterly certification but maintained their privileges this finding will be escalated to senior management if the issue is not remediated."
+SUS.IAMS.4.2.5.7 (p.18): "Access is denied if any of the minimum required reviewers (workforce member's management ...) deny access to a workforce member."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+SUS.IAMS.4.2.5.6 (p.17): "Managers shall be responsible for attesting to the entitlements and roles assigned to their direct employees, contractors, and other workforce members. Application Owners shall be responsible for attesting to the entitlements of vendor, system, and uncorrelated accounts."</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Removal not sustained; re-grant and new ISEAdmin membership approved without requests; account not linked to an HR identity in SanIAM.</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Requests + approvals for the re-grant and ISEAdmin add; correlate to SanIAM identity.</t>
         </is>
@@ -765,12 +812,25 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: The 2025 Q3 removal met the 30-business-day SLA (4.2.5.21), but PAM Proc. 4.1.1 C4 and 4.2 require that revoked access stays removed and that retained access is escalated - it was back in AD by 11/25/2025 with no escalation. Under 4.2.5.7 the manager's denial means access is denied; giving it back required a new documented request, manager validation and second-level approval (4.2.3.4). None exists, yet the access was approved again on 4/30/2026.
+Also: not correlated to an HR identity (4.2.1.1, 4.2.5.6); new ISEAdmin membership without request (4.2.3.4).
+IAM Std v10.0 SUS.IAMS.4.2.5.21 (p.22): "Any revocation of privileged access rights resulting from the privileged access review outcomes shall be completed within 30 business days of the close of the review."
+PAM Procedure v2.0 sec. 4.1.1 C4 (p.6): "When the ServiceNow ticket is closed, the PAM Team confirms that access is de-provisioned correctly."
+PAM Procedure v2.0 sec. 4.2 (p.7): "If PAM US Team identifies that a user whose access was rejected during a quarterly certification but maintained their privileges this finding will be escalated to senior management if the issue is not remediated."
+SUS.IAMS.4.2.5.7 (p.18): "Access is denied if any of the minimum required reviewers (workforce member's management ...) deny access to a workforce member."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+SUS.IAMS.4.2.5.6 (p.17): "Managers shall be responsible for attesting to the entitlements and roles assigned to their direct employees, contractors, and other workforce members. Application Owners shall be responsible for attesting to the entitlements of vendor, system, and uncorrelated accounts."</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Removal not sustained; re-grant and new ISEAdmin membership approved without requests; account not linked to an HR identity.</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Requests + approvals for the re-grant and ISEAdmin add; correlate to SanIAM identity.</t>
         </is>
@@ -830,12 +890,22 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: The 2025 Q3 removal met the 30-business-day SLA (4.2.5.21), but PAM Proc. 4.1.1 C4 and 4.2 require that revoked access stays removed and that retained access is escalated - it was back in AD by 11/25/2025 with no escalation. Under 4.2.5.7 the manager's denial means access is denied; giving it back required a new documented request, manager validation and second-level approval (4.2.3.4). None exists, yet the access was approved again on 4/30/2026.
+IAM Std v10.0 SUS.IAMS.4.2.5.21 (p.22): "Any revocation of privileged access rights resulting from the privileged access review outcomes shall be completed within 30 business days of the close of the review."
+PAM Procedure v2.0 sec. 4.1.1 C4 (p.6): "When the ServiceNow ticket is closed, the PAM Team confirms that access is de-provisioned correctly."
+PAM Procedure v2.0 sec. 4.2 (p.7): "If PAM US Team identifies that a user whose access was rejected during a quarterly certification but maintained their privileges this finding will be escalated to senior management if the issue is not remediated."
+SUS.IAMS.4.2.5.7 (p.18): "Access is denied if any of the minimum required reviewers (workforce member's management ...) deny access to a workforce member."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Revocation timely but not sustained; re-grant approved without a request.</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>Approved ServiceNow request + Netwrix 'member added' event for the re-grant.</t>
         </is>
@@ -895,12 +965,22 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: 4.2.5.1 requires the review to confirm that access remains valid and follows least privilege. Privileged CISCO/ISE admin access on an AD account disabled and unused since 10/15/2023 is not valid or needed, yet it was approved on 8/28/2025 and 4/30/2026. 4.2.3.1 requires accounts unused for 90 days to be disabled or removed - the account was disabled but its privileged group memberships were kept and re-certified. Fieldglass satisfies 4.2.1.1 (HR is authoritative - active contractor), so the termination-date issue is cleared, but that does not cure the approval of inactive access. SLA (4.2.5.21) not applicable - nothing was revoked (process owner position agreed, PAM step 9).
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+SUS.IAMS.4.2.3.1 (p.10): "User Active Directory accounts unused for the previous 90 calendar days shall be reviewed for inactivity and, if confirmed to be inactive, disabled or removed."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+IAM Std v10.0 SUS.IAMS.4.2.5.21 (p.22): "Any revocation of privileged access rights resulting from the privileged access review outcomes shall be completed within 30 business days of the close of the review."
+PAM Procedure v2.0 sec. 8 step 9 (p.10): "When all assignees have completed their decisions, if the manager approves the user access, the process ends. If access is revoked, the PAM team submits revocation tickets for any 'reject' decision or terminated users."</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Fieldglass shows he is an active contractor, but privileged admin access unused for ~2 years on a disabled account is not valid or needed (4.2.5.1); inactive accounts must be disabled or removed (4.2.3.1). The reviewer should have revoked it - exception in both samples.</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Recommend revocation; unlikely to clear.</t>
         </is>
@@ -960,12 +1040,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT PASSES: 4.2.1.1 makes HR the authoritative source for external users - for contractors that is Fieldglass. Fieldglass shows worker SANWK00016508 Open 2024-01-01 to 2027-02-28, covering both decision dates (8/28/2025, 4/30/2026), so the SanIAM 12/31/2024 termination date is stale and the user was not a leaver. 4.2.5.6 makes the manager responsible for attesting contractors' entitlements - the line manager approved in both semi-annual samples. The account was enabled and in use, so the access remained valid (4.2.5.1). No revocation occurred, so the SLA in 4.2.5.21 is not triggered (PAM step 9: if the manager approves, the process ends).
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+SUS.IAMS.4.2.5.6 (p.17): "Managers shall be responsible for attesting to the entitlements and roles assigned to their direct employees, contractors, and other workforce members. Application Owners shall be responsible for attesting to the entitlements of vendor, system, and uncorrelated accounts."
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+PAM Procedure v2.0 sec. 8 step 9 (p.10): "When all assignees have completed their decisions, if the manager approves the user access, the process ends. If access is revoked, the PAM team submits revocation tickets for any 'reject' decision or terminated users."</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Fieldglass shows an open engagement on both decision dates, so 12/31/2024 is stale SanIAM data, not a termination. Active, enabled account approved by the line manager (4.2.5.6). No exception.</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -1025,12 +1114,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT PASSES: Fieldglass (HR authoritative source, 4.2.1.1) shows worker SANWK00016502 Open 2024-01-01 to 2027-02-28 - active on both decision dates; the IAMS 12/31/2024 date is stale. Manager attested an active, enabled contractor in both samples (4.2.5.6, 4.2.5.1). No revocation - SLA not triggered (4.2.5.21; PAM step 9).
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+SUS.IAMS.4.2.5.6 (p.17): "Managers shall be responsible for attesting to the entitlements and roles assigned to their direct employees, contractors, and other workforce members. Application Owners shall be responsible for attesting to the entitlements of vendor, system, and uncorrelated accounts."
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+PAM Procedure v2.0 sec. 8 step 9 (p.10): "When all assignees have completed their decisions, if the manager approves the user access, the process ends. If access is revoked, the PAM team submits revocation tickets for any 'reject' decision or terminated users."</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Fieldglass clears the termination-date issue; approved access of an active, enabled contractor in both samples. No exception.</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -1090,12 +1188,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT PASSES: Fieldglass (HR authoritative source, 4.2.1.1) shows worker SANWK00016503 Open 2024-01-01 to 2027-02-28 - active on both decision dates; the IAMS 12/31/2024 date is stale. Manager attested an active, enabled contractor in both samples (4.2.5.6, 4.2.5.1). No revocation - SLA not triggered (4.2.5.21; PAM step 9).
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."
+SUS.IAMS.4.2.5.6 (p.17): "Managers shall be responsible for attesting to the entitlements and roles assigned to their direct employees, contractors, and other workforce members. Application Owners shall be responsible for attesting to the entitlements of vendor, system, and uncorrelated accounts."
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+PAM Procedure v2.0 sec. 8 step 9 (p.10): "When all assignees have completed their decisions, if the manager approves the user access, the process ends. If access is revoked, the PAM team submits revocation tickets for any 'reject' decision or terminated users."</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Fieldglass clears the termination-date issue; approved access of an active, enabled contractor in both samples. No exception.</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>FAIL only if Fieldglass detail shows a lapse on a decision date.</t>
         </is>
@@ -1155,12 +1262,21 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: 2025 Q3 passes - Fieldglass (4.2.1.1) shows an Open engagement and the account was enabled and in use. In 2026 Q1, 4.2.5.1 required the reviewer to confirm the access remained valid; the account had been disabled in AD since 4/2/2026, yet its privileged access was approved on 4/30/2026 without the disabled status being addressed. The account was later re-enabled with no request or approval, contrary to 4.2.3.4. Fieldglass shows he was not terminated, but does not explain the disablement.
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+SUS.IAMS.4.2.3.1 (p.10): "User Active Directory accounts unused for the previous 90 calendar days shall be reviewed for inactivity and, if confirmed to be inactive, disabled or removed."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>2025 Q3 passes. 2026 Q1 fails: privileged access approved on an account disabled since 4/2/2026; the later re-enable is unevidenced.</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Reason for the 4/2-4/3/2026 disablement of 9 contractor accounts + approved re-enable request could reduce to an observation.</t>
         </is>
@@ -1220,12 +1336,21 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>WHY IT FAILS: 2025 Q3 passes - Fieldglass (4.2.1.1) shows an Open engagement. In 2026 Q1 privileged access was approved on 4/30/2026 for an account disabled in AD since 4/3/2026 without the reviewer addressing it (4.2.5.1); the later re-enable has no request or approval (4.2.3.4). Also: blank AD employeeNumber - the account is not fully synchronized with HR (4.2.1.1).
+SUS.IAMS.4.2.5.1 (p.14): "The recertification process shall be performed as a formal review of information assets to confirm that all granted access rights entitlements remain valid, updated, and in full compliance with the SoD rules and Principle of Least Privilege."
+SUS.IAMS.4.2.3.1 (p.10): "User Active Directory accounts unused for the previous 90 calendar days shall be reviewed for inactivity and, if confirmed to be inactive, disabled or removed."
+SUS.IAMS.4.2.3.4 (p.11): "Access rights must be provisioned only when requested by an Access Requestor via an approved request mechanism, validated by the proper manager, and authorized by a second level approver ... The use of an approved mechanism is required to confirm that the request and approval is fully documented for auditing purposes."
+SUS.IAMS.4.2.1.1 (p.6-7): "For external users, HR shall be the authoritative source for all external user account information." / "Personal accounts must be fully synchronized with Santander US HR Systems."</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>2025 Q3 passes. 2026 Q1 fails: access approved on an account disabled since 4/3/2026; re-enable unevidenced; blank employeeNumber.</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Same as MIA25249; also populate employeeNumber.</t>
         </is>
@@ -1273,10 +1398,17 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Policy quotes are from IAM Standard v10.0 (approved 09/29/2025, in force for both samples; same requirement IDs and substance in v11.0 approved 07/28/2026) and BSI PAM Recertification Procedure v2.0 (04/22/2026). Page numbers refer to v10.0.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M14"/>
+  <autoFilter ref="A4:N14"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>